<commit_message>
Redraw flowchart with standard notation: ○ start/end, ◇ branch, □ action
開始/終了に楕円○、判断分岐にひし形◇、処理に四角□の標準記号を使用。

https://claude.ai/code/session_014LN5dU5LtPSyG4iXygZNs3
</commit_message>
<xml_diff>
--- a/LPN分割_誤り対応フロー図.xlsx
+++ b/LPN分割_誤り対応フロー図.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="誤り対応フロー図" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LPN分割誤り対応フロー" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -133,7 +133,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="13335000" cy="9734550"/>
+    <ext cx="13335000" cy="10058400"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>

</xml_diff>

<commit_message>
Fix missing r: namespace in sheet1.xml causing Excel to reject the file
https://claude.ai/code/session_014LN5dU5LtPSyG4iXygZNs3
</commit_message>
<xml_diff>
--- a/LPN分割_誤り対応フロー図.xlsx
+++ b/LPN分割_誤り対応フロー図.xlsx
@@ -2270,5 +2270,24 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><sheetPr><outlinePr summaryBelow="1" summaryRight="1" /><pageSetUpPr /></sheetPr><dimension ref="A1:A1" /><sheetFormatPr baseColWidth="8" defaultRowHeight="15" /><sheetData><row r="1" ht="20" customHeight="1"><c r="A1" s="1" t="inlineStr"><is><t>LPN分割 誤り対応フロー図</t></is></c></row></sheetData><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5" /><drawing r:id="rId10"/></worksheet>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LPN分割 誤り対応フロー図</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId10"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix shape positioning: calculate col/row properly from COL_EMU/ROW_EMU
colOffが列幅を超えていたため全図形が左上に重なっていた問題を修正。
列幅・行高を固定してcol/rowを正しく算出するよう変更。

https://claude.ai/code/session_014LN5dU5LtPSyG4iXygZNs3
</commit_message>
<xml_diff>
--- a/LPN分割_誤り対応フロー図.xlsx
+++ b/LPN分割_誤り対応フロー図.xlsx
@@ -190,10 +190,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>648000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>306000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="9525" cy="126000"/>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>52000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9525" cy="125999"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="3" name="Conn3"/>
@@ -202,7 +202,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9525" cy="126000"/>
+          <a:ext cx="9525" cy="125999"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -221,8 +221,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>432000</xdr:rowOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>178000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="396000"/>
     <xdr:sp macro="" textlink="">
@@ -283,10 +283,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1188000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>630000</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>521250</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>122000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="360000" cy="9525"/>
     <xdr:cxnSp macro="">
@@ -314,10 +314,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1548000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>396000</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>214500</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>142000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1296000" cy="468000"/>
     <xdr:sp macro="" textlink="">
@@ -377,12 +377,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2844000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>630000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="396000" cy="9525"/>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>177000</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>122000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="395999" cy="9525"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="7" name="Conn7"/>
@@ -391,7 +391,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="396000" cy="9525"/>
+          <a:ext cx="395999" cy="9525"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -408,10 +408,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2862000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>522000</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>195000</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>14000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="288000" cy="144000"/>
     <xdr:sp macro="" textlink="">
@@ -456,10 +456,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>3240000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>468000</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>573000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>214000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1260000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -508,10 +508,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2196000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>864000</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>195750</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>102000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="252000"/>
     <xdr:cxnSp macro="">
@@ -539,10 +539,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2232000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>936000</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>231750</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>174000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="251999" cy="125999"/>
     <xdr:sp macro="" textlink="">
@@ -587,10 +587,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1548000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1116000</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>214500</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>100000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1296000" cy="468000"/>
     <xdr:sp macro="" textlink="">
@@ -650,12 +650,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2844000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1350000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="396000" cy="9525"/>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>177000</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>80000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="395999" cy="9525"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="13" name="Conn13"/>
@@ -664,7 +664,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="396000" cy="9525"/>
+          <a:ext cx="395999" cy="9525"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -681,10 +681,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2862000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1242000</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>195000</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>226000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="360000" cy="144000"/>
     <xdr:sp macro="" textlink="">
@@ -729,10 +729,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>3240000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1188000</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>573000</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>172000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1260000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -792,10 +792,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2196000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1584000</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>195750</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>60000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="251999"/>
     <xdr:cxnSp macro="">
@@ -823,10 +823,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2232000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1638000</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>231750</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>114000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="396000" cy="125999"/>
     <xdr:sp macro="" textlink="">
@@ -871,10 +871,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1548000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1835999</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>214500</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>57999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1296000" cy="396000"/>
     <xdr:sp macro="" textlink="">
@@ -936,10 +936,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>2520000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="4680000" cy="9525"/>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>234000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4860000" cy="9525"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="19" name="Sep19"/>
@@ -948,7 +948,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="4680000" cy="9525"/>
+          <a:ext cx="4860000" cy="9525"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -967,8 +967,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>2592000</xdr:rowOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>52000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="234000"/>
     <xdr:sp macro="" textlink="">
@@ -1021,8 +1021,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>648000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>2826000</xdr:rowOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>32000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="125999"/>
     <xdr:cxnSp macro="">
@@ -1052,8 +1052,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>2951999</xdr:rowOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>157999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -1114,10 +1114,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1188000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>3114000</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>521250</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>66000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="432000" cy="9525"/>
     <xdr:cxnSp macro="">
@@ -1145,10 +1145,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1620000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>2951999</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>286500</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>157999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1260000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -1199,10 +1199,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>3600000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="4680000" cy="9525"/>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>44000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4860000" cy="9525"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="25" name="Sep25"/>
@@ -1211,7 +1211,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="4680000" cy="9525"/>
+          <a:ext cx="4860000" cy="9525"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1230,8 +1230,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>3671999</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>115999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="234000"/>
     <xdr:sp macro="" textlink="">
@@ -1284,8 +1284,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>648000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>3906000</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>96000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="125999"/>
     <xdr:cxnSp macro="">
@@ -1315,8 +1315,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>4031999</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>221999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -1377,10 +1377,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1188000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>4194000</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>521250</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>130000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="432000" cy="9525"/>
     <xdr:cxnSp macro="">
@@ -1408,10 +1408,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1620000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>4031999</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>286500</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>221999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1260000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -1462,10 +1462,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>4680000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="4680000" cy="9525"/>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>108000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4860000" cy="9525"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="31" name="Sep31"/>
@@ -1474,7 +1474,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="4680000" cy="9525"/>
+          <a:ext cx="4860000" cy="9525"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1493,8 +1493,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>4752000</xdr:rowOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>180000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="234000"/>
     <xdr:sp macro="" textlink="">
@@ -1547,10 +1547,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>648000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>4986000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="9525" cy="126000"/>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>160000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9525" cy="125999"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="33" name="Conn33"/>
@@ -1559,7 +1559,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9525" cy="126000"/>
+          <a:ext cx="9525" cy="125999"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1578,8 +1578,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>5112000</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>32000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="360000"/>
     <xdr:sp macro="" textlink="">
@@ -1640,10 +1640,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1188000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>5292000</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>521250</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>212000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="432000" cy="9525"/>
     <xdr:cxnSp macro="">
@@ -1671,10 +1671,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1620000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>5112000</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>286500</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>32000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1260000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -1725,10 +1725,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>5760000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="4680000" cy="9525"/>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>172000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4860000" cy="9525"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="37" name="Sep37"/>
@@ -1737,7 +1737,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="4680000" cy="9525"/>
+          <a:ext cx="4860000" cy="9525"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1756,8 +1756,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>5832000</xdr:rowOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>244000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="234000"/>
     <xdr:sp macro="" textlink="">
@@ -1810,10 +1810,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>648000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>6066000</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="9525" cy="126000"/>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>224000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9525" cy="125999"/>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
         <xdr:cNvPr id="39" name="Conn39"/>
@@ -1822,7 +1822,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9525" cy="126000"/>
+          <a:ext cx="9525" cy="125999"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1841,8 +1841,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>108000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>6192000</xdr:rowOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>96000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1080000" cy="360000"/>
     <xdr:sp macro="" textlink="">
@@ -1903,10 +1903,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1188000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>6372000</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>521250</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>22000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="432000" cy="9525"/>
     <xdr:cxnSp macro="">
@@ -1934,10 +1934,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1620000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>6192000</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>286500</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>96000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1260000" cy="324000"/>
     <xdr:sp macro="" textlink="">
@@ -2278,6 +2278,29 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+  </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
@@ -2286,6 +2309,64 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="20" customHeight="1"/>
+    <row r="3" ht="20" customHeight="1"/>
+    <row r="4" ht="20" customHeight="1"/>
+    <row r="5" ht="20" customHeight="1"/>
+    <row r="6" ht="20" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1"/>
+    <row r="8" ht="20" customHeight="1"/>
+    <row r="9" ht="20" customHeight="1"/>
+    <row r="10" ht="20" customHeight="1"/>
+    <row r="11" ht="20" customHeight="1"/>
+    <row r="12" ht="20" customHeight="1"/>
+    <row r="13" ht="20" customHeight="1"/>
+    <row r="14" ht="20" customHeight="1"/>
+    <row r="15" ht="20" customHeight="1"/>
+    <row r="16" ht="20" customHeight="1"/>
+    <row r="17" ht="20" customHeight="1"/>
+    <row r="18" ht="20" customHeight="1"/>
+    <row r="19" ht="20" customHeight="1"/>
+    <row r="20" ht="20" customHeight="1"/>
+    <row r="21" ht="20" customHeight="1"/>
+    <row r="22" ht="20" customHeight="1"/>
+    <row r="23" ht="20" customHeight="1"/>
+    <row r="24" ht="20" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1"/>
+    <row r="26" ht="20" customHeight="1"/>
+    <row r="27" ht="20" customHeight="1"/>
+    <row r="28" ht="20" customHeight="1"/>
+    <row r="29" ht="20" customHeight="1"/>
+    <row r="30" ht="20" customHeight="1"/>
+    <row r="31" ht="20" customHeight="1"/>
+    <row r="32" ht="20" customHeight="1"/>
+    <row r="33" ht="20" customHeight="1"/>
+    <row r="34" ht="20" customHeight="1"/>
+    <row r="35" ht="20" customHeight="1"/>
+    <row r="36" ht="20" customHeight="1"/>
+    <row r="37" ht="20" customHeight="1"/>
+    <row r="38" ht="20" customHeight="1"/>
+    <row r="39" ht="20" customHeight="1"/>
+    <row r="40" ht="20" customHeight="1"/>
+    <row r="41" ht="20" customHeight="1"/>
+    <row r="42" ht="20" customHeight="1"/>
+    <row r="43" ht="20" customHeight="1"/>
+    <row r="44" ht="20" customHeight="1"/>
+    <row r="45" ht="20" customHeight="1"/>
+    <row r="46" ht="20" customHeight="1"/>
+    <row r="47" ht="20" customHeight="1"/>
+    <row r="48" ht="20" customHeight="1"/>
+    <row r="49" ht="20" customHeight="1"/>
+    <row r="50" ht="20" customHeight="1"/>
+    <row r="51" ht="20" customHeight="1"/>
+    <row r="52" ht="20" customHeight="1"/>
+    <row r="53" ht="20" customHeight="1"/>
+    <row r="54" ht="20" customHeight="1"/>
+    <row r="55" ht="20" customHeight="1"/>
+    <row r="56" ht="20" customHeight="1"/>
+    <row r="57" ht="20" customHeight="1"/>
+    <row r="58" ht="20" customHeight="1"/>
+    <row r="59" ht="20" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId10"/>

</xml_diff>